<commit_message>
fixed lat lonf and qty
</commit_message>
<xml_diff>
--- a/pds_admin_mizoram/Backend/Backend/Data_2.xlsx
+++ b/pds_admin_mizoram/Backend/Backend/Data_2.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="363">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="386">
   <si>
     <t>SW_ID</t>
   </si>
@@ -1088,22 +1088,91 @@
     <t>Storage_Capacity</t>
   </si>
   <si>
-    <t>Anjawc</t>
-  </si>
-  <si>
-    <t>WC16048bbbhhh</t>
-  </si>
-  <si>
-    <t>MSWC</t>
-  </si>
-  <si>
-    <t>27.99097</t>
-  </si>
-  <si>
-    <t>96.73109</t>
-  </si>
-  <si>
-    <t>6767</t>
+    <t>Fd15003</t>
+  </si>
+  <si>
+    <t>Fd15001</t>
+  </si>
+  <si>
+    <t>Fd15005</t>
+  </si>
+  <si>
+    <t>Fd15002</t>
+  </si>
+  <si>
+    <t>Fd15004</t>
+  </si>
+  <si>
+    <t>Fd15007</t>
+  </si>
+  <si>
+    <t>FD15003</t>
+  </si>
+  <si>
+    <t>FD15001</t>
+  </si>
+  <si>
+    <t>FD15005</t>
+  </si>
+  <si>
+    <t>FD15002</t>
+  </si>
+  <si>
+    <t>FD15004</t>
+  </si>
+  <si>
+    <t>FD15007</t>
+  </si>
+  <si>
+    <t>fci</t>
+  </si>
+  <si>
+    <t>23.73833314</t>
+  </si>
+  <si>
+    <t>24.24627618</t>
+  </si>
+  <si>
+    <t>24.1007769</t>
+  </si>
+  <si>
+    <t>22.86601579</t>
+  </si>
+  <si>
+    <t>24.2012396</t>
+  </si>
+  <si>
+    <t>22.52471726</t>
+  </si>
+  <si>
+    <t>92.67722146</t>
+  </si>
+  <si>
+    <t>92.68273129</t>
+  </si>
+  <si>
+    <t>92.68498096</t>
+  </si>
+  <si>
+    <t>92.74049945</t>
+  </si>
+  <si>
+    <t>92.54186875</t>
+  </si>
+  <si>
+    <t>92.91176285</t>
+  </si>
+  <si>
+    <t>574200</t>
+  </si>
+  <si>
+    <t>626400</t>
+  </si>
+  <si>
+    <t>365400</t>
+  </si>
+  <si>
+    <t>417600</t>
   </si>
 </sst>
 </file>
@@ -3731,7 +3800,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -3768,19 +3837,134 @@
         <v>357</v>
       </c>
       <c r="D2" t="s">
+        <v>363</v>
+      </c>
+      <c r="E2" t="s">
+        <v>369</v>
+      </c>
+      <c r="F2" t="s">
+        <v>370</v>
+      </c>
+      <c r="G2" t="s">
+        <v>376</v>
+      </c>
+      <c r="H2" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="B3" t="s">
+        <v>120</v>
+      </c>
+      <c r="C3" t="s">
         <v>358</v>
       </c>
-      <c r="E2" t="s">
+      <c r="D3" t="s">
+        <v>364</v>
+      </c>
+      <c r="E3" t="s">
+        <v>369</v>
+      </c>
+      <c r="F3" t="s">
+        <v>371</v>
+      </c>
+      <c r="G3" t="s">
+        <v>377</v>
+      </c>
+      <c r="H3" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="B4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C4" t="s">
         <v>359</v>
       </c>
-      <c r="F2" t="s">
+      <c r="D4" t="s">
+        <v>365</v>
+      </c>
+      <c r="E4" t="s">
+        <v>369</v>
+      </c>
+      <c r="F4" t="s">
+        <v>372</v>
+      </c>
+      <c r="G4" t="s">
+        <v>378</v>
+      </c>
+      <c r="H4" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="B5" t="s">
+        <v>127</v>
+      </c>
+      <c r="C5" t="s">
         <v>360</v>
       </c>
-      <c r="G2" t="s">
+      <c r="D5" t="s">
+        <v>366</v>
+      </c>
+      <c r="E5" t="s">
+        <v>369</v>
+      </c>
+      <c r="F5" t="s">
+        <v>373</v>
+      </c>
+      <c r="G5" t="s">
+        <v>379</v>
+      </c>
+      <c r="H5" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="B6" t="s">
+        <v>120</v>
+      </c>
+      <c r="C6" t="s">
         <v>361</v>
       </c>
-      <c r="H2" t="s">
+      <c r="D6" t="s">
+        <v>367</v>
+      </c>
+      <c r="E6" t="s">
+        <v>369</v>
+      </c>
+      <c r="F6" t="s">
+        <v>374</v>
+      </c>
+      <c r="G6" t="s">
+        <v>380</v>
+      </c>
+      <c r="H6" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="B7" t="s">
+        <v>124</v>
+      </c>
+      <c r="C7" t="s">
         <v>362</v>
+      </c>
+      <c r="D7" t="s">
+        <v>368</v>
+      </c>
+      <c r="E7" t="s">
+        <v>369</v>
+      </c>
+      <c r="F7" t="s">
+        <v>375</v>
+      </c>
+      <c r="G7" t="s">
+        <v>381</v>
+      </c>
+      <c r="H7" t="s">
+        <v>385</v>
       </c>
     </row>
   </sheetData>

</xml_diff>